<commit_message>
Ajout d'un valueset ruleset et d'un codesystem ruleset (ShareableValueSet / ShareableCodeSystem & language fr-FR) (#277)
* add valueset ruleset

* update

* pudate

* update cs

* error

* update

* update b86237b4ce4eff8e5bb8ca6675ff43bdc5ed72e2
</commit_message>
<xml_diff>
--- a/main/ig/CodeSystem-fr-core-cs-champ-activite.xlsx
+++ b/main/ig/CodeSystem-fr-core-cs-champ-activite.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="59">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-23T09:26:22+00:00</t>
+    <t>2026-02-23T10:39:10+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -147,16 +147,31 @@
     <t>MCO</t>
   </si>
   <si>
+    <t>Médecine Chirurgie Obstétrique</t>
+  </si>
+  <si>
     <t>SMR</t>
   </si>
   <si>
+    <t>Soins Médicaux et de Réadaptation</t>
+  </si>
+  <si>
     <t>HAD</t>
   </si>
   <si>
+    <t>Hospitalisation à Domicile</t>
+  </si>
+  <si>
     <t>PSY</t>
   </si>
   <si>
+    <t>Psychiatrie</t>
+  </si>
+  <si>
     <t>EHPAD</t>
+  </si>
+  <si>
+    <t>Etablissement d'Hébergement pour Personnes Agées Dépendantes</t>
   </si>
   <si>
     <t>LG_SJR</t>
@@ -519,91 +534,107 @@
       <c r="C2" t="s" s="2">
         <v>43</v>
       </c>
-      <c r="D2" s="2"/>
+      <c r="D2" t="s" s="2">
+        <v>44</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
         <v>42</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>44</v>
-      </c>
-      <c r="D3" s="2"/>
+        <v>45</v>
+      </c>
+      <c r="D3" t="s" s="2">
+        <v>46</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
         <v>42</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>45</v>
-      </c>
-      <c r="D4" s="2"/>
+        <v>47</v>
+      </c>
+      <c r="D4" t="s" s="2">
+        <v>48</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
         <v>42</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>46</v>
-      </c>
-      <c r="D5" s="2"/>
+        <v>49</v>
+      </c>
+      <c r="D5" t="s" s="2">
+        <v>50</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
         <v>42</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C6" t="s" s="2">
-        <v>47</v>
-      </c>
-      <c r="D6" s="2"/>
+        <v>51</v>
+      </c>
+      <c r="D6" t="s" s="2">
+        <v>52</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
         <v>42</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C7" t="s" s="2">
-        <v>49</v>
-      </c>
-      <c r="D7" s="2"/>
+        <v>54</v>
+      </c>
+      <c r="D7" t="s" s="2">
+        <v>54</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
         <v>42</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C8" t="s" s="2">
-        <v>51</v>
-      </c>
-      <c r="D8" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="D8" t="s" s="2">
+        <v>56</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
         <v>42</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C9" t="s" s="2">
-        <v>53</v>
-      </c>
-      <c r="D9" s="2"/>
+        <v>58</v>
+      </c>
+      <c r="D9" t="s" s="2">
+        <v>58</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
Update jurisdiction label in sushi-config.yaml 5f5cd199020cbb3cc54d08ffb6f93e7cfd2e69ec
</commit_message>
<xml_diff>
--- a/main/ig/CodeSystem-fr-core-cs-champ-activite.xlsx
+++ b/main/ig/CodeSystem-fr-core-cs-champ-activite.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-25T15:00:47+00:00</t>
+    <t>2026-03-31T09:16:18+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,7 @@
     <t>Jurisdiction</t>
   </si>
   <si>
-    <t>France</t>
+    <t>France (la)</t>
   </si>
   <si>
     <t>Description</t>

</xml_diff>